<commit_message>
Updated inventory forecasting model and dataset support
</commit_message>
<xml_diff>
--- a/data/CV1.xlsx
+++ b/data/CV1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maanya\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Maanya\ClaimVerification\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C009F398-3716-43FA-AB88-8202068F1994}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDC3F6F6-D4D4-4E52-B405-97B9F4548B28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{1A1D6C68-4408-46F7-8369-2AD15A3E1D72}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="64">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="96">
   <si>
     <t>FG CODE</t>
   </si>
@@ -231,6 +231,102 @@
   </si>
   <si>
     <t>https://www.myntra.com/40388973</t>
+  </si>
+  <si>
+    <t>40AC805340</t>
+  </si>
+  <si>
+    <t>Polo</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/32008231</t>
+  </si>
+  <si>
+    <t>40BC236002</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/33194405</t>
+  </si>
+  <si>
+    <t>40BC236111</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/37938959</t>
+  </si>
+  <si>
+    <t>40BM105001</t>
+  </si>
+  <si>
+    <t>Shirt</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/32106413</t>
+  </si>
+  <si>
+    <t>40BM105230</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/32106414</t>
+  </si>
+  <si>
+    <t>40BM108110</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/35190805</t>
+  </si>
+  <si>
+    <t>40BM127062</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/36228999</t>
+  </si>
+  <si>
+    <t>40BM127280</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/36229000</t>
+  </si>
+  <si>
+    <t>40BM333001</t>
+  </si>
+  <si>
+    <t>CKJM</t>
+  </si>
+  <si>
+    <t>Sweater</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/34741710</t>
+  </si>
+  <si>
+    <t>Regular</t>
+  </si>
+  <si>
+    <t>Regular Fit</t>
+  </si>
+  <si>
+    <t>CLASSIC</t>
+  </si>
+  <si>
+    <t>Slim</t>
+  </si>
+  <si>
+    <t>40BM343001</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/36654183</t>
+  </si>
+  <si>
+    <t>40BM343811</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/36078101</t>
+  </si>
+  <si>
+    <t>40BM347001</t>
+  </si>
+  <si>
+    <t>https://www.myntra.com/36078103</t>
   </si>
 </sst>
 </file>
@@ -288,7 +384,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -296,19 +392,6 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -655,7 +738,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E28B301-CBD8-4311-B664-D813A20757D5}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -974,22 +1057,22 @@
       <c r="A13">
         <v>0</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" t="s">
         <v>49</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="D13" s="7" t="s">
+      <c r="D13" t="s">
         <v>50</v>
       </c>
-      <c r="E13" s="9">
+      <c r="E13" s="3">
         <v>35950255</v>
       </c>
-      <c r="F13" s="8" t="s">
+      <c r="F13" t="s">
         <v>51</v>
       </c>
-      <c r="G13" s="9" t="s">
+      <c r="G13" s="3" t="s">
         <v>52</v>
       </c>
       <c r="H13">
@@ -1001,22 +1084,22 @@
       <c r="A14">
         <v>0</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" t="s">
         <v>53</v>
       </c>
-      <c r="C14" s="11" t="s">
+      <c r="C14" t="s">
         <v>57</v>
       </c>
-      <c r="D14" s="12" t="s">
+      <c r="D14" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="13">
+      <c r="E14" s="3">
         <v>35190831</v>
       </c>
-      <c r="F14" s="12" t="s">
+      <c r="F14" t="s">
         <v>58</v>
       </c>
-      <c r="G14" s="13" t="s">
+      <c r="G14" s="3" t="s">
         <v>59</v>
       </c>
       <c r="H14">
@@ -1027,22 +1110,22 @@
       <c r="A15">
         <v>0</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" t="s">
         <v>54</v>
       </c>
-      <c r="C15" s="11" t="s">
+      <c r="C15" t="s">
         <v>57</v>
       </c>
-      <c r="D15" s="12" t="s">
+      <c r="D15" t="s">
         <v>50</v>
       </c>
-      <c r="E15" s="13">
+      <c r="E15" s="3">
         <v>35190823</v>
       </c>
-      <c r="F15" s="12" t="s">
+      <c r="F15" t="s">
         <v>60</v>
       </c>
-      <c r="G15" s="13" t="s">
+      <c r="G15" s="3" t="s">
         <v>59</v>
       </c>
       <c r="H15">
@@ -1053,22 +1136,22 @@
       <c r="A16">
         <v>0</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" t="s">
         <v>55</v>
       </c>
-      <c r="C16" s="11" t="s">
+      <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="12" t="s">
+      <c r="D16" t="s">
         <v>50</v>
       </c>
-      <c r="E16" s="13">
+      <c r="E16" s="3">
         <v>39247554</v>
       </c>
-      <c r="F16" s="12" t="s">
+      <c r="F16" t="s">
         <v>61</v>
       </c>
-      <c r="G16" s="13" t="s">
+      <c r="G16" s="3" t="s">
         <v>62</v>
       </c>
       <c r="H16">
@@ -1079,26 +1162,338 @@
       <c r="A17">
         <v>0</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" t="s">
         <v>56</v>
       </c>
-      <c r="C17" s="11" t="s">
+      <c r="C17" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="12" t="s">
+      <c r="D17" t="s">
         <v>50</v>
       </c>
-      <c r="E17" s="13">
+      <c r="E17" s="3">
         <v>40388973</v>
       </c>
-      <c r="F17" s="12" t="s">
+      <c r="F17" t="s">
         <v>63</v>
       </c>
-      <c r="G17" s="13" t="s">
+      <c r="G17" s="3" t="s">
         <v>52</v>
       </c>
       <c r="H17">
         <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18">
+        <v>0</v>
+      </c>
+      <c r="B18" t="s">
+        <v>64</v>
+      </c>
+      <c r="C18" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" t="s">
+        <v>65</v>
+      </c>
+      <c r="E18">
+        <v>32008231</v>
+      </c>
+      <c r="F18" t="s">
+        <v>66</v>
+      </c>
+      <c r="G18">
+        <v>0</v>
+      </c>
+      <c r="H18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19">
+        <v>0</v>
+      </c>
+      <c r="B19" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" t="s">
+        <v>20</v>
+      </c>
+      <c r="D19" t="s">
+        <v>65</v>
+      </c>
+      <c r="E19">
+        <v>33194405</v>
+      </c>
+      <c r="F19" t="s">
+        <v>68</v>
+      </c>
+      <c r="G19">
+        <v>0</v>
+      </c>
+      <c r="H19" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20">
+        <v>0</v>
+      </c>
+      <c r="B20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C20" t="s">
+        <v>20</v>
+      </c>
+      <c r="D20" t="s">
+        <v>65</v>
+      </c>
+      <c r="E20">
+        <v>37938959</v>
+      </c>
+      <c r="F20" t="s">
+        <v>70</v>
+      </c>
+      <c r="G20">
+        <v>0</v>
+      </c>
+      <c r="H20" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>0</v>
+      </c>
+      <c r="B21" t="s">
+        <v>71</v>
+      </c>
+      <c r="C21" t="s">
+        <v>20</v>
+      </c>
+      <c r="D21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E21">
+        <v>32106413</v>
+      </c>
+      <c r="F21" t="s">
+        <v>73</v>
+      </c>
+      <c r="G21">
+        <v>0</v>
+      </c>
+      <c r="H21" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>0</v>
+      </c>
+      <c r="B22" t="s">
+        <v>74</v>
+      </c>
+      <c r="C22" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" t="s">
+        <v>72</v>
+      </c>
+      <c r="E22">
+        <v>32106414</v>
+      </c>
+      <c r="F22" t="s">
+        <v>75</v>
+      </c>
+      <c r="G22">
+        <v>0</v>
+      </c>
+      <c r="H22" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>0</v>
+      </c>
+      <c r="B23" t="s">
+        <v>76</v>
+      </c>
+      <c r="C23" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" t="s">
+        <v>72</v>
+      </c>
+      <c r="E23">
+        <v>35190805</v>
+      </c>
+      <c r="F23" t="s">
+        <v>77</v>
+      </c>
+      <c r="G23">
+        <v>0</v>
+      </c>
+      <c r="H23" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>0</v>
+      </c>
+      <c r="B24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C24" t="s">
+        <v>20</v>
+      </c>
+      <c r="D24" t="s">
+        <v>72</v>
+      </c>
+      <c r="E24">
+        <v>36228999</v>
+      </c>
+      <c r="F24" t="s">
+        <v>79</v>
+      </c>
+      <c r="G24">
+        <v>0</v>
+      </c>
+      <c r="H24" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>0</v>
+      </c>
+      <c r="B25" t="s">
+        <v>80</v>
+      </c>
+      <c r="C25" t="s">
+        <v>20</v>
+      </c>
+      <c r="D25" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25">
+        <v>36229000</v>
+      </c>
+      <c r="F25" t="s">
+        <v>81</v>
+      </c>
+      <c r="G25">
+        <v>0</v>
+      </c>
+      <c r="H25" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>0</v>
+      </c>
+      <c r="B26" t="s">
+        <v>82</v>
+      </c>
+      <c r="C26" t="s">
+        <v>83</v>
+      </c>
+      <c r="D26" t="s">
+        <v>84</v>
+      </c>
+      <c r="E26">
+        <v>34741710</v>
+      </c>
+      <c r="F26" t="s">
+        <v>85</v>
+      </c>
+      <c r="G26">
+        <v>0</v>
+      </c>
+      <c r="H26" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A27">
+        <v>0</v>
+      </c>
+      <c r="B27" t="s">
+        <v>90</v>
+      </c>
+      <c r="C27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D27" t="s">
+        <v>84</v>
+      </c>
+      <c r="E27">
+        <v>36654183</v>
+      </c>
+      <c r="F27" t="s">
+        <v>91</v>
+      </c>
+      <c r="G27">
+        <v>0</v>
+      </c>
+      <c r="H27" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A28">
+        <v>0</v>
+      </c>
+      <c r="B28" t="s">
+        <v>92</v>
+      </c>
+      <c r="C28" t="s">
+        <v>20</v>
+      </c>
+      <c r="D28" t="s">
+        <v>84</v>
+      </c>
+      <c r="E28">
+        <v>36078101</v>
+      </c>
+      <c r="F28" t="s">
+        <v>93</v>
+      </c>
+      <c r="G28">
+        <v>0</v>
+      </c>
+      <c r="H28" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A29">
+        <v>0</v>
+      </c>
+      <c r="B29" t="s">
+        <v>94</v>
+      </c>
+      <c r="C29" t="s">
+        <v>20</v>
+      </c>
+      <c r="D29" t="s">
+        <v>84</v>
+      </c>
+      <c r="E29">
+        <v>36078103</v>
+      </c>
+      <c r="F29" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="G29">
+        <v>0</v>
+      </c>
+      <c r="H29" t="s">
+        <v>87</v>
       </c>
     </row>
   </sheetData>
@@ -1109,6 +1504,7 @@
     <hyperlink ref="F2" r:id="rId1" xr:uid="{3AAFCE4D-1980-420E-A8C0-CB62F59A328F}"/>
     <hyperlink ref="F4:F5" r:id="rId2" display="https://www.myntra.com/38551423" xr:uid="{D9EEABA5-CF9E-41CA-8B17-72A3AC084302}"/>
     <hyperlink ref="F5:F12" r:id="rId3" display="https://www.myntra.com/38551423" xr:uid="{5D0F30B1-140B-4EA8-A262-1211323688D8}"/>
+    <hyperlink ref="F29" r:id="rId4" xr:uid="{46A8916E-5341-4478-989C-A98AD24A494C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>